<commit_message>
fix(ba-kit): template_estimation không lưu tên file 見積書 nguồn (có tên khách hàng)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ba-kit/system-to-doc/templates/template_estimation.xlsx
+++ b/ba-kit/system-to-doc/templates/template_estimation.xlsx
@@ -17,11 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy&quot;/&quot;mm&quot;/&quot;dd"/>
-    <numFmt numFmtId="166" formatCode="\¥#,##0_);[Red]&quot;(¥&quot;#,##0\)"/>
-    <numFmt numFmtId="167" formatCode="\¥#,##0_);&quot;(¥&quot;#,##0\)"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy&quot;/&quot;mm&quot;/&quot;dd"/>
+    <numFmt numFmtId="165" formatCode="\¥#,##0_);[Red]&quot;(¥&quot;#,##0\)"/>
+    <numFmt numFmtId="166" formatCode="\¥#,##0_);&quot;(¥&quot;#,##0\)"/>
   </numFmts>
   <fonts count="25">
     <font>
@@ -206,7 +205,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="35">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -511,11 +510,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="dotted">
+        <color rgb="FF4BACC6"/>
+      </left>
+      <right/>
+      <top style="dotted">
+        <color rgb="FF4BACC6"/>
+      </top>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -583,7 +592,7 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="12" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -598,13 +607,13 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="15" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="15" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="15" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -782,6 +791,18 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1195,7 +1216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI237"/>
+  <dimension ref="A1:AH237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.71" customWidth="1" min="1" max="1"/>
@@ -1566,7 +1587,7 @@
           <t>■見積日</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="96" t="inlineStr">
         <is>
           <t>{{DATE}}</t>
         </is>
@@ -1610,7 +1631,7 @@
           <t>■有効期限</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="96" t="inlineStr">
         <is>
           <t>{{VALID_UNTIL}}</t>
         </is>
@@ -1726,13 +1747,13 @@
           <t>合計金額（税別）</t>
         </is>
       </c>
-      <c r="D15" s="28" t="n"/>
+      <c r="D15" s="97" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="n"/>
       <c r="H15" s="6" t="n"/>
       <c r="I15" s="6" t="n"/>
       <c r="J15" s="29" t="n"/>
-      <c r="K15" s="30" t="n"/>
+      <c r="K15" s="98" t="n"/>
       <c r="O15" s="31" t="n"/>
       <c r="P15" s="31" t="n"/>
       <c r="Q15" s="5" t="n"/>
@@ -2290,7 +2311,7 @@
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="1" t="n"/>
-      <c r="B28" s="74" t="inlineStr">
+      <c r="B28" s="99" t="inlineStr">
         <is>
           <t>◆前提条件</t>
         </is>
@@ -9899,7 +9920,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>【TOKIWAGI様】見積書_団体利用_2609.xlsx</t>
+          <t>見積書 (ten file nguon khong luu — co ten khach hang)</t>
         </is>
       </c>
     </row>

</xml_diff>